<commit_message>
fix: to correct the planifiction for week 1
</commit_message>
<xml_diff>
--- a/doc/planification/planification.xlsx
+++ b/doc/planification/planification.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://eduvaud-my.sharepoint.com/personal/pi11mws_eduvaud_ch/Documents/Documents/Obsidian Vault/Diplôme/dossier finale travail de diplôme/archive annexes/planification/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\edepierr\programmation\.github\doc\planification\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="455" documentId="13_ncr:1_{EDC051C4-9A1E-4E2D-8F43-8C514157D3AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6115EF3A-00FA-481E-8662-49D3055E79EA}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DB0E887-DD86-4887-8A8D-BE08D0F26A0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{82FCF275-8522-428A-8299-FE516CA6C369}"/>
   </bookViews>
@@ -18,7 +18,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">dashboard!$B$2:$G$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'to do'!$A$1:$G$71</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'to do'!$A$1:$G$67</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
   <extLst>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="73">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="81">
   <si>
     <t>achèvement</t>
   </si>
@@ -121,21 +121,9 @@
     <t xml:space="preserve">faire la page front de d'authentification simple </t>
   </si>
   <si>
-    <t xml:space="preserve">faire la partie back d'authentification simple </t>
-  </si>
-  <si>
     <t>Authentification / inscription</t>
   </si>
   <si>
-    <t xml:space="preserve">faire la page front de l'enregistrement simple </t>
-  </si>
-  <si>
-    <t xml:space="preserve">faire la partie back de l'enregistrement simple </t>
-  </si>
-  <si>
-    <t>faire la page d'accueil initial</t>
-  </si>
-  <si>
     <t xml:space="preserve">Ecrire le template de la definition of done </t>
   </si>
   <si>
@@ -154,9 +142,6 @@
     <t>conception du diagramme de micro-service</t>
   </si>
   <si>
-    <t>faire les différent dashboard de rôle</t>
-  </si>
-  <si>
     <t>total</t>
   </si>
   <si>
@@ -172,33 +157,6 @@
     <t xml:space="preserve">faire la liste des restaurant front  </t>
   </si>
   <si>
-    <t xml:space="preserve">documenter la fonctionnalité commande dans le rapport </t>
-  </si>
-  <si>
-    <t>faire la partie gestion du compte front (CRUD) (clients)</t>
-  </si>
-  <si>
-    <t>faire la partie gestion du compte back (CRUD) (clients)</t>
-  </si>
-  <si>
-    <t>faire la partie gestion du compte front (CRUD) (restaurant partenaire)</t>
-  </si>
-  <si>
-    <t>faire la partie gestion du compte back (CRUD) (restaurant partenaire)</t>
-  </si>
-  <si>
-    <t>faire la partie gestion du compte front (CRUD) (modérateur)</t>
-  </si>
-  <si>
-    <t>faire la partie gestion du compte back (CRUD) (modérateur)</t>
-  </si>
-  <si>
-    <t>faire la partie gestion du compte back (CRUD) (administrateur)</t>
-  </si>
-  <si>
-    <t>faire la partie gestion du compte front (CRUD) (administrateur)</t>
-  </si>
-  <si>
     <t>Sprints</t>
   </si>
   <si>
@@ -259,10 +217,76 @@
     <t>lire les consigne cahier des charges et écouter à la séance d'information</t>
   </si>
   <si>
-    <t>faire la partie gestion du compte front (CRUD) (livreur)</t>
-  </si>
-  <si>
-    <t>faire la partie gestion du compte back (CRUD) (livreur)</t>
+    <t>faire la partie gestion du compte front create user</t>
+  </si>
+  <si>
+    <t>faire la partie gestion du compte back create user</t>
+  </si>
+  <si>
+    <t>faire la partie gestion du compte front delete user</t>
+  </si>
+  <si>
+    <t>faire la partie gestion du compte back delete user</t>
+  </si>
+  <si>
+    <t>faire la partie gestion du compte front modify user</t>
+  </si>
+  <si>
+    <t>faire la partie gestion du compte back modify user</t>
+  </si>
+  <si>
+    <t>faire la partie gestion du compte back lecture user</t>
+  </si>
+  <si>
+    <t>faire les différent dashboard de rôle (livreur et user)</t>
+  </si>
+  <si>
+    <t>faire les différent dashboard de rôle (modérateur et admin)</t>
+  </si>
+  <si>
+    <t>faire la partie gestion du compte front lecture user</t>
+  </si>
+  <si>
+    <t xml:space="preserve">documenter la fonctionnalité livraison dans le rapport </t>
+  </si>
+  <si>
+    <t>documenter la gestion de rôle</t>
+  </si>
+  <si>
+    <t xml:space="preserve">faire les différent dashboard de rôle (restaurateur) </t>
+  </si>
+  <si>
+    <t>faire la partie authentification complète</t>
+  </si>
+  <si>
+    <t>faire le diagramme de séquence de la fonctionnalité</t>
+  </si>
+  <si>
+    <t>Mettre à jour la documentation pour correspondre à l'ajout</t>
+  </si>
+  <si>
+    <t>Objectif</t>
+  </si>
+  <si>
+    <t>Mettre en place l'environnement</t>
+  </si>
+  <si>
+    <t>Authentification et gestion de compte (page d'accueil par type de compte)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conclure le rapport </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Commande fonctionnelle </t>
+  </si>
+  <si>
+    <t>Conclure le rapport</t>
+  </si>
+  <si>
+    <t>Livraison fonctionnelle  + modification de la gestion de compte</t>
+  </si>
+  <si>
+    <t>Faire la partie gestion du restaurant</t>
   </si>
 </sst>
 </file>
@@ -307,7 +331,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="20">
+  <borders count="24">
     <border>
       <left/>
       <right/>
@@ -525,12 +549,36 @@
       <diagonal/>
     </border>
     <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
@@ -538,14 +586,14 @@
       <diagonal/>
     </border>
     <border>
-      <left style="medium">
+      <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top/>
-      <bottom style="medium">
+      <right/>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -554,9 +602,7 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top/>
       <bottom style="medium">
         <color indexed="64"/>
@@ -564,13 +610,45 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -581,7 +659,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1">
@@ -630,19 +708,23 @@
     <xf numFmtId="9" fontId="0" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="9" fontId="2" fillId="0" borderId="15" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="9" fontId="2" fillId="0" borderId="16" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="2" fontId="0" fillId="2" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="19" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="2" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="18" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="1" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="20" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="21" xfId="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1067,6 +1149,7 @@
     <col min="2" max="2" width="44.7109375" customWidth="1"/>
     <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
     <col min="4" max="7" width="14.85546875" customWidth="1"/>
+    <col min="8" max="8" width="63.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
@@ -1090,8 +1173,8 @@
         <v>4</v>
       </c>
       <c r="I2" s="27">
-        <f>COUNTIF('to do'!$G$3:G$2024,TRUE)/(COUNTIF('to do'!$G$3:G$2024,TRUE)+COUNTIF('to do'!$G$3:G$2024,FALSE))</f>
-        <v>0.15942028985507245</v>
+        <f>COUNTIF('to do'!$G$3:G$2020,TRUE)/(COUNTIF('to do'!$G$3:G$2020,TRUE)+COUNTIF('to do'!$G$3:G$2020,FALSE))</f>
+        <v>0.2</v>
       </c>
     </row>
     <row r="3" spans="2:9" x14ac:dyDescent="0.25">
@@ -1099,15 +1182,15 @@
         <v>11</v>
       </c>
       <c r="C3" s="19">
-        <f>COUNTIFS('to do'!$A$3:$A$524,B3,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$A$3:$A$524,B3)</f>
+        <f>COUNTIFS('to do'!$A$3:$A$520,B3,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$A$3:$A$520,B3)</f>
         <v>1</v>
       </c>
       <c r="D3" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B3,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$A$2:$A$520,B3,'to do'!D$2:D$20041)</f>
         <v>4.25</v>
       </c>
       <c r="E3" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B3,'to do'!E$2:E$20045)</f>
+        <f>SUMIF('to do'!$A$2:$A$520,B3,'to do'!E$2:E$20041)</f>
         <v>4.25</v>
       </c>
       <c r="F3" s="21">
@@ -1115,7 +1198,7 @@
       </c>
       <c r="G3" s="22">
         <f t="shared" ref="G3:G10" ca="1" si="0">F3-TODAY()</f>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4" spans="2:9" x14ac:dyDescent="0.25">
@@ -1123,15 +1206,15 @@
         <v>12</v>
       </c>
       <c r="C4" s="6">
-        <f>COUNTIFS('to do'!$A$3:$A$524,B4,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$A$3:$A$524,B4)</f>
+        <f>COUNTIFS('to do'!$A$3:$A$520,B4,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$A$3:$A$520,B4)</f>
         <v>1</v>
       </c>
       <c r="D4" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B4,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$A$2:$A$520,B4,'to do'!D$2:D$20041)</f>
         <v>8.25</v>
       </c>
       <c r="E4" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B4,'to do'!E$2:E$20045)</f>
+        <f>SUMIF('to do'!$A$2:$A$520,B4,'to do'!E$2:E$20041)</f>
         <v>8.25</v>
       </c>
       <c r="F4" s="3">
@@ -1139,31 +1222,31 @@
       </c>
       <c r="G4" s="16">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B5" s="15" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C5" s="6">
-        <f>COUNTIFS('to do'!$A$3:$A$524,B5,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$A$3:$A$524,B5)</f>
-        <v>0</v>
+        <f>COUNTIFS('to do'!$A$3:$A$520,B5,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$A$3:$A$520,B5)</f>
+        <v>0.5</v>
       </c>
       <c r="D5" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B5,'to do'!D$2:D$20045)</f>
-        <v>0</v>
+        <f>SUMIF('to do'!$A$2:$A$520,B5,'to do'!D$2:D$20041)</f>
+        <v>2.25</v>
       </c>
       <c r="E5" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B5,'to do'!E$2:E$20045)</f>
-        <v>10</v>
+        <f>SUMIF('to do'!$A$2:$A$520,B5,'to do'!E$2:E$20041)</f>
+        <v>4</v>
       </c>
       <c r="F5" s="3">
         <v>46255</v>
       </c>
       <c r="G5" s="16">
         <f t="shared" ca="1" si="0"/>
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6" spans="2:9" x14ac:dyDescent="0.25">
@@ -1171,23 +1254,23 @@
         <v>13</v>
       </c>
       <c r="C6" s="6">
-        <f>COUNTIFS('to do'!$A$3:$A$524,B6,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$A$3:$A$524,B6)</f>
+        <f>COUNTIFS('to do'!$A$3:$A$520,B6,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$A$3:$A$520,B6)</f>
         <v>0.21428571428571427</v>
       </c>
       <c r="D6" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B6,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$A$2:$A$520,B6,'to do'!D$2:D$20041)</f>
         <v>7.5</v>
       </c>
       <c r="E6" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B6,'to do'!E$2:E$20045)</f>
-        <v>39.5</v>
+        <f>SUMIF('to do'!$A$2:$A$520,B6,'to do'!E$2:E$20041)</f>
+        <v>26.5</v>
       </c>
       <c r="F6" s="3">
         <v>46262</v>
       </c>
       <c r="G6" s="16">
         <f t="shared" ca="1" si="0"/>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="2:9" x14ac:dyDescent="0.25">
@@ -1195,23 +1278,23 @@
         <v>16</v>
       </c>
       <c r="C7" s="6">
-        <f>COUNTIFS('to do'!$A$3:$A$524,B7,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$A$3:$A$524,B7)</f>
+        <f>COUNTIFS('to do'!$A$3:$A$520,B7,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$A$3:$A$520,B7)</f>
         <v>0</v>
       </c>
       <c r="D7" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B7,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$A$2:$A$520,B7,'to do'!D$2:D$20041)</f>
         <v>0</v>
       </c>
       <c r="E7" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B7,'to do'!E$2:E$20045)</f>
-        <v>16</v>
+        <f>SUMIF('to do'!$A$2:$A$520,B7,'to do'!E$2:E$20041)</f>
+        <v>8</v>
       </c>
       <c r="F7" s="3">
         <v>46262</v>
       </c>
       <c r="G7" s="16">
         <f ca="1">F7-TODAY()</f>
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="2:9" x14ac:dyDescent="0.25">
@@ -1219,23 +1302,23 @@
         <v>15</v>
       </c>
       <c r="C8" s="6">
-        <f>COUNTIFS('to do'!$A$3:$A$524,B8,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$A$3:$A$524,B8)</f>
+        <f>COUNTIFS('to do'!$A$3:$A$520,B8,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$A$3:$A$520,B8)</f>
         <v>0</v>
       </c>
       <c r="D8" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B8,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$A$2:$A$520,B8,'to do'!D$2:D$20041)</f>
         <v>0</v>
       </c>
       <c r="E8" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B8,'to do'!E$2:E$20045)</f>
-        <v>32</v>
+        <f>SUMIF('to do'!$A$2:$A$520,B8,'to do'!E$2:E$20041)</f>
+        <v>31</v>
       </c>
       <c r="F8" s="3">
         <v>46276</v>
       </c>
       <c r="G8" s="16">
         <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H8" s="8"/>
     </row>
@@ -1244,61 +1327,61 @@
         <v>14</v>
       </c>
       <c r="C9" s="6">
-        <f>COUNTIFS('to do'!$A$3:$A$524,B9,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$A$3:$A$524,B9)</f>
+        <f>COUNTIFS('to do'!$A$3:$A$520,B9,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$A$3:$A$520,B9)</f>
         <v>0</v>
       </c>
       <c r="D9" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B9,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$A$2:$A$520,B9,'to do'!D$2:D$20041)</f>
         <v>0</v>
       </c>
       <c r="E9" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B9,'to do'!E$2:E$20045)</f>
-        <v>32</v>
+        <f>SUMIF('to do'!$A$2:$A$520,B9,'to do'!E$2:E$20041)</f>
+        <v>26</v>
       </c>
       <c r="F9" s="3">
         <v>46283</v>
       </c>
       <c r="G9" s="16">
         <f t="shared" ca="1" si="0"/>
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="10" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B10" s="17" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="C10" s="9">
-        <f>COUNTIFS('to do'!$A$3:$A$524,B10,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$A$3:$A$524,B10)</f>
-        <v>0</v>
+        <f>COUNTIFS('to do'!$A$3:$A$520,B10,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$A$3:$A$520,B10)</f>
+        <v>0.25</v>
       </c>
       <c r="D10" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B10,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$A$2:$A$520,B10,'to do'!D$2:D$20041)</f>
         <v>2</v>
       </c>
       <c r="E10" s="20">
-        <f>SUMIF('to do'!$A$2:$A$524,B10,'to do'!E$2:E$20045)</f>
-        <v>28</v>
+        <f>SUMIF('to do'!$A$2:$A$520,B10,'to do'!E$2:E$20041)</f>
+        <v>42</v>
       </c>
       <c r="F10" s="10">
         <v>46283</v>
       </c>
       <c r="G10" s="18">
         <f t="shared" ca="1" si="0"/>
-        <v>29</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="B11" s="11" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C11" s="12"/>
       <c r="D11" s="13">
         <f>SUM(D3:D10)</f>
-        <v>22</v>
+        <v>24.25</v>
       </c>
       <c r="E11" s="13">
         <f>SUM(E3:E10)</f>
-        <v>170</v>
+        <v>150</v>
       </c>
       <c r="F11" s="12"/>
       <c r="G11" s="14"/>
@@ -1306,7 +1389,7 @@
     <row r="12" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="13" spans="2:9" x14ac:dyDescent="0.25">
       <c r="B13" s="28" t="s">
-        <v>51</v>
+        <v>37</v>
       </c>
       <c r="C13" s="29" t="s">
         <v>0</v>
@@ -1318,147 +1401,166 @@
         <v>2</v>
       </c>
       <c r="F13" s="29" t="s">
-        <v>52</v>
-      </c>
-      <c r="G13" s="30" t="s">
+        <v>38</v>
+      </c>
+      <c r="G13" s="35" t="s">
         <v>4</v>
       </c>
+      <c r="H13" s="38" t="s">
+        <v>73</v>
+      </c>
     </row>
     <row r="14" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B14" s="35">
+      <c r="B14" s="33">
         <v>0</v>
       </c>
       <c r="C14" s="6">
-        <f>COUNTIFS('to do'!$C$3:$C$524,B14,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$C$3:$C$524,B14)</f>
-        <v>0.6470588235294118</v>
+        <f>COUNTIFS('to do'!$C$3:$C$520,B14,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$C$3:$C$520,B14)</f>
+        <v>0.9285714285714286</v>
       </c>
       <c r="D14" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B14,'to do'!D$2:D$20045)</f>
-        <v>22</v>
+        <f>SUMIF('to do'!$C$2:$C$520,B14,'to do'!D$2:D$20041)</f>
+        <v>24.25</v>
       </c>
       <c r="E14" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B14,'to do'!E$2:E$20045)</f>
-        <v>34</v>
+        <f>SUMIF('to do'!$C$2:$C$520,B14,'to do'!E$2:E$20041)</f>
+        <v>28</v>
       </c>
       <c r="F14" s="3">
         <v>46255</v>
       </c>
-      <c r="G14" s="16">
+      <c r="G14" s="36">
         <f t="shared" ref="G14:G18" ca="1" si="1">F14-TODAY()</f>
-        <v>1</v>
+        <v>0</v>
+      </c>
+      <c r="H14" s="39" t="s">
+        <v>74</v>
       </c>
     </row>
     <row r="15" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B15" s="36">
+      <c r="B15" s="34">
         <v>1</v>
       </c>
       <c r="C15" s="6">
-        <f>COUNTIFS('to do'!$C$3:$C$524,B15,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$C$3:$C$524,B15)</f>
+        <f>COUNTIFS('to do'!$C$3:$C$520,B15,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$C$3:$C$520,B15)</f>
         <v>0</v>
       </c>
       <c r="D15" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B15,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$C$2:$C$520,B15,'to do'!D$2:D$20041)</f>
         <v>0</v>
       </c>
       <c r="E15" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B15,'to do'!E$2:E$20045)</f>
-        <v>36</v>
+        <f>SUMIF('to do'!$C$2:$C$520,B15,'to do'!E$2:E$20041)</f>
+        <v>30</v>
       </c>
       <c r="F15" s="3">
         <v>46262</v>
       </c>
-      <c r="G15" s="16">
+      <c r="G15" s="36">
         <f t="shared" ca="1" si="1"/>
-        <v>8</v>
+        <v>7</v>
+      </c>
+      <c r="H15" s="39" t="s">
+        <v>75</v>
       </c>
     </row>
     <row r="16" spans="2:9" x14ac:dyDescent="0.25">
-      <c r="B16" s="36">
+      <c r="B16" s="34">
         <v>2</v>
       </c>
       <c r="C16" s="6">
-        <f>COUNTIFS('to do'!$C$3:$C$524,B16,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$C$3:$C$524,B16)</f>
+        <f>COUNTIFS('to do'!$C$3:$C$520,B16,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$C$3:$C$520,B16)</f>
         <v>0</v>
       </c>
       <c r="D16" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B16,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$C$2:$C$520,B16,'to do'!D$2:D$20041)</f>
         <v>0</v>
       </c>
       <c r="E16" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B16,'to do'!E$2:E$20045)</f>
-        <v>34</v>
+        <f>SUMIF('to do'!$C$2:$C$520,B16,'to do'!E$2:E$20041)</f>
+        <v>32</v>
       </c>
       <c r="F16" s="3">
         <v>46269</v>
       </c>
-      <c r="G16" s="16">
+      <c r="G16" s="36">
         <f t="shared" ca="1" si="1"/>
-        <v>15</v>
-      </c>
-    </row>
-    <row r="17" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B17" s="36">
+        <v>14</v>
+      </c>
+      <c r="H16" s="39" t="s">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B17" s="34">
         <v>3</v>
       </c>
       <c r="C17" s="6">
-        <f>COUNTIFS('to do'!$C$3:$C$524,B17,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$C$3:$C$524,B17)</f>
+        <f>COUNTIFS('to do'!$C$3:$C$520,B17,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$C$3:$C$520,B17)</f>
         <v>0</v>
       </c>
       <c r="D17" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B17,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$C$2:$C$520,B17,'to do'!D$2:D$20041)</f>
         <v>0</v>
       </c>
       <c r="E17" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B17,'to do'!E$2:E$20045)</f>
-        <v>34</v>
+        <f>SUMIF('to do'!$C$2:$C$520,B17,'to do'!E$2:E$20041)</f>
+        <v>30</v>
       </c>
       <c r="F17" s="3">
         <v>46276</v>
       </c>
-      <c r="G17" s="16">
+      <c r="G17" s="36">
         <f t="shared" ca="1" si="1"/>
-        <v>22</v>
-      </c>
-    </row>
-    <row r="18" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B18" s="36">
+        <v>21</v>
+      </c>
+      <c r="H17" s="39" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="B18" s="34">
         <v>4</v>
       </c>
       <c r="C18" s="6">
-        <f>COUNTIFS('to do'!$C$3:$C$524,B18,'to do'!$G$3:$G$524,TRUE)/COUNTIF('to do'!$C$3:$C$524,B18)</f>
+        <f>COUNTIFS('to do'!$C$3:$C$520,B18,'to do'!$G$3:$G$520,TRUE)/COUNTIF('to do'!$C$3:$C$520,B18)</f>
         <v>0</v>
       </c>
       <c r="D18" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B18,'to do'!D$2:D$20045)</f>
+        <f>SUMIF('to do'!$C$2:$C$520,B18,'to do'!D$2:D$20041)</f>
         <v>0</v>
       </c>
       <c r="E18" s="7">
-        <f>SUMIF('to do'!$C$2:$C$524,B18,'to do'!E$2:E$20045)</f>
-        <v>32</v>
+        <f>SUMIF('to do'!$C$2:$C$520,B18,'to do'!E$2:E$20041)</f>
+        <v>30</v>
       </c>
       <c r="F18" s="3">
         <v>46283</v>
       </c>
-      <c r="G18" s="16">
+      <c r="G18" s="36">
         <f t="shared" ca="1" si="1"/>
-        <v>29</v>
-      </c>
-    </row>
-    <row r="19" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B19" s="31" t="s">
-        <v>37</v>
-      </c>
-      <c r="C19" s="32"/>
-      <c r="D19" s="33">
+        <v>28</v>
+      </c>
+      <c r="H18" s="39" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="19" spans="2:8" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B19" s="30" t="s">
+        <v>32</v>
+      </c>
+      <c r="C19" s="31"/>
+      <c r="D19" s="32">
         <f>SUM(D12:D18)</f>
-        <v>22</v>
-      </c>
-      <c r="E19" s="33">
+        <v>24.25</v>
+      </c>
+      <c r="E19" s="32">
         <f>SUM(E14:E18)</f>
-        <v>170</v>
-      </c>
-      <c r="F19" s="32"/>
-      <c r="G19" s="34"/>
+        <v>150</v>
+      </c>
+      <c r="F19" s="31"/>
+      <c r="G19" s="37"/>
+      <c r="H19" s="40"/>
     </row>
   </sheetData>
   <autoFilter ref="B2:G11" xr:uid="{595B6011-1975-4F59-9917-E41DFA55B94C}"/>
@@ -1526,11 +1628,11 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{515B20D0-7813-4B7C-85BE-27293B2A524B}">
   <sheetPr filterMode="1"/>
-  <dimension ref="A1:G75"/>
+  <dimension ref="A1:G67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="38.28515625" customWidth="1"/>
-    <col min="2" max="2" width="72.85546875" style="5" customWidth="1"/>
+    <col min="2" max="2" width="72.5703125" style="5" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21.5703125" style="5" customWidth="1"/>
     <col min="4" max="5" width="16.5703125" style="5" customWidth="1"/>
     <col min="6" max="6" width="31.5703125" customWidth="1"/>
@@ -1564,7 +1666,7 @@
         <v>11</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>70</v>
+        <v>56</v>
       </c>
       <c r="C2" s="4">
         <v>0</v>
@@ -1685,9 +1787,9 @@
         <v>1</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
-        <v>67</v>
+        <v>53</v>
       </c>
       <c r="B8" s="4" t="s">
         <v>23</v>
@@ -1703,12 +1805,12 @@
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B9" s="4" t="s">
         <v>24</v>
@@ -1716,21 +1818,23 @@
       <c r="C9" s="4">
         <v>0</v>
       </c>
-      <c r="D9" s="4"/>
+      <c r="D9" s="4">
+        <v>2.25</v>
+      </c>
       <c r="E9" s="4">
         <v>2</v>
       </c>
       <c r="F9" s="1"/>
       <c r="G9" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>25</v>
+        <v>70</v>
       </c>
       <c r="C10" s="4">
         <v>0</v>
@@ -1744,12 +1848,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="B11" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="C11" s="4">
         <v>0</v>
@@ -1760,58 +1864,64 @@
       </c>
       <c r="F11" s="1"/>
       <c r="G11" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B12" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C12" s="4">
         <v>0</v>
       </c>
-      <c r="D12" s="4"/>
+      <c r="D12" s="4">
+        <v>3</v>
+      </c>
       <c r="E12" s="4">
         <v>2</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4" t="s">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="B13" s="4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C13" s="4">
         <v>0</v>
       </c>
-      <c r="D13" s="4"/>
+      <c r="D13" s="4">
+        <v>3.5</v>
+      </c>
       <c r="E13" s="4">
-        <v>2</v>
+        <v>3.5</v>
       </c>
       <c r="F13" s="1"/>
       <c r="G13" s="2" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="14" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="C14" s="4">
         <v>0</v>
       </c>
-      <c r="D14" s="4"/>
+      <c r="D14" s="4">
+        <v>1</v>
+      </c>
       <c r="E14" s="4">
         <v>2</v>
       </c>
@@ -1822,16 +1932,16 @@
     </row>
     <row r="15" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>33</v>
+        <v>30</v>
       </c>
       <c r="C15" s="4">
         <v>0</v>
       </c>
       <c r="D15" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E15" s="4">
         <v>2</v>
@@ -1843,7 +1953,7 @@
     </row>
     <row r="16" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B16" s="4" t="s">
         <v>31</v>
@@ -1852,145 +1962,139 @@
         <v>0</v>
       </c>
       <c r="D16" s="4">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="E16" s="4">
-        <v>3.5</v>
+        <v>2</v>
       </c>
       <c r="F16" s="1"/>
       <c r="G16" s="2" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A17" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B17" s="4" t="s">
-        <v>32</v>
+        <v>64</v>
       </c>
       <c r="C17" s="4">
-        <v>0</v>
-      </c>
-      <c r="D17" s="4">
-        <v>1</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D17" s="4"/>
       <c r="E17" s="4">
         <v>2</v>
       </c>
       <c r="F17" s="1"/>
       <c r="G17" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A18" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B18" s="4" t="s">
-        <v>34</v>
+        <v>57</v>
       </c>
       <c r="C18" s="4">
-        <v>0</v>
-      </c>
-      <c r="D18" s="4">
-        <v>2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D18" s="4"/>
       <c r="E18" s="4">
         <v>2</v>
       </c>
       <c r="F18" s="1"/>
       <c r="G18" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A19" s="4" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B19" s="4" t="s">
-        <v>35</v>
+        <v>58</v>
       </c>
       <c r="C19" s="4">
-        <v>0</v>
-      </c>
-      <c r="D19" s="4">
-        <v>2</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D19" s="4"/>
       <c r="E19" s="4">
         <v>2</v>
       </c>
       <c r="F19" s="1"/>
       <c r="G19" s="2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A20" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>36</v>
+        <v>59</v>
       </c>
       <c r="C20" s="4">
         <v>1</v>
       </c>
       <c r="D20" s="4"/>
       <c r="E20" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F20" s="1"/>
       <c r="G20" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A21" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B21" s="4" t="s">
-        <v>43</v>
+        <v>60</v>
       </c>
       <c r="C21" s="4">
         <v>1</v>
       </c>
       <c r="D21" s="4"/>
       <c r="E21" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F21" s="1"/>
       <c r="G21" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A22" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>44</v>
+        <v>61</v>
       </c>
       <c r="C22" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D22" s="4"/>
       <c r="E22" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F22" s="1"/>
       <c r="G22" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>45</v>
+        <v>62</v>
       </c>
       <c r="C23" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D23" s="4"/>
       <c r="E23" s="4">
@@ -2001,34 +2105,34 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A24" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>46</v>
+        <v>66</v>
       </c>
       <c r="C24" s="4">
         <v>1</v>
       </c>
       <c r="D24" s="4"/>
       <c r="E24" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F24" s="1"/>
       <c r="G24" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>47</v>
+        <v>63</v>
       </c>
       <c r="C25" s="4">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D25" s="4"/>
       <c r="E25" s="4">
@@ -2039,69 +2143,69 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B26" s="4" t="s">
-        <v>48</v>
+        <v>65</v>
       </c>
       <c r="C26" s="4">
         <v>1</v>
       </c>
       <c r="D26" s="4"/>
       <c r="E26" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F26" s="1"/>
       <c r="G26" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
         <v>13</v>
       </c>
       <c r="B27" s="4" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="C27" s="4">
         <v>1</v>
       </c>
       <c r="D27" s="4"/>
       <c r="E27" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F27" s="1"/>
       <c r="G27" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B28" s="4" t="s">
-        <v>49</v>
+        <v>41</v>
       </c>
       <c r="C28" s="4">
         <v>1</v>
       </c>
       <c r="D28" s="4"/>
       <c r="E28" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F28" s="1"/>
       <c r="G28" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B29" s="4" t="s">
-        <v>71</v>
+        <v>39</v>
       </c>
       <c r="C29" s="4">
         <v>1</v>
@@ -2115,110 +2219,110 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B30" s="4" t="s">
-        <v>72</v>
+        <v>40</v>
       </c>
       <c r="C30" s="4">
         <v>1</v>
       </c>
       <c r="D30" s="4"/>
       <c r="E30" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F30" s="1"/>
       <c r="G30" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A31" s="4" t="s">
         <v>16</v>
       </c>
       <c r="B31" s="4" t="s">
-        <v>55</v>
+        <v>42</v>
       </c>
       <c r="C31" s="4">
         <v>1</v>
       </c>
       <c r="D31" s="4"/>
       <c r="E31" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F31" s="1"/>
       <c r="G31" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B32" s="4" t="s">
-        <v>53</v>
+        <v>33</v>
       </c>
       <c r="C32" s="4">
         <v>2</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F32" s="1"/>
       <c r="G32" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="33" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A33" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B33" s="4" t="s">
-        <v>54</v>
+        <v>34</v>
       </c>
       <c r="C33" s="4">
         <v>2</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F33" s="1"/>
       <c r="G33" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B34" s="4" t="s">
-        <v>56</v>
+        <v>36</v>
       </c>
       <c r="C34" s="4">
         <v>2</v>
       </c>
       <c r="D34" s="4"/>
       <c r="E34" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F34" s="1"/>
       <c r="G34" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A35" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="C35" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D35" s="4"/>
       <c r="E35" s="4">
@@ -2229,53 +2333,53 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B36" s="4" t="s">
-        <v>39</v>
+        <v>51</v>
       </c>
       <c r="C36" s="4">
         <v>2</v>
       </c>
       <c r="D36" s="4"/>
       <c r="E36" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F36" s="1"/>
       <c r="G36" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="37" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A37" s="4" t="s">
         <v>15</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>41</v>
+        <v>52</v>
       </c>
       <c r="C37" s="4">
         <v>2</v>
       </c>
       <c r="D37" s="4"/>
       <c r="E37" s="4">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F37" s="1"/>
       <c r="G37" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="B38" s="4" t="s">
-        <v>40</v>
+        <v>68</v>
       </c>
       <c r="C38" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D38" s="4"/>
       <c r="E38" s="4">
@@ -2286,91 +2390,91 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A39" s="4" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="B39" s="4" t="s">
-        <v>65</v>
+        <v>78</v>
       </c>
       <c r="C39" s="4">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D39" s="4"/>
       <c r="E39" s="4">
-        <v>8</v>
+        <v>30</v>
       </c>
       <c r="F39" s="1"/>
       <c r="G39" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>15</v>
+        <v>53</v>
       </c>
       <c r="B40" s="4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="C40" s="4">
         <v>3</v>
       </c>
       <c r="D40" s="4"/>
       <c r="E40" s="4">
-        <v>8</v>
+        <v>4</v>
       </c>
       <c r="F40" s="1"/>
       <c r="G40" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A41" s="4" t="s">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="B41" s="4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="C41" s="4">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D41" s="4"/>
       <c r="E41" s="4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F41" s="1"/>
       <c r="G41" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="B42" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C42" s="4">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D42" s="4"/>
       <c r="E42" s="4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F42" s="1"/>
       <c r="G42" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A43" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B43" s="4" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C43" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D43" s="4"/>
       <c r="E43" s="4">
@@ -2381,91 +2485,91 @@
         <v>0</v>
       </c>
     </row>
-    <row r="44" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B44" s="4" t="s">
-        <v>57</v>
+        <v>50</v>
       </c>
       <c r="C44" s="4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D44" s="4"/>
       <c r="E44" s="4">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="F44" s="1"/>
       <c r="G44" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A45" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B45" s="4" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="C45" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D45" s="4"/>
       <c r="E45" s="4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F45" s="1"/>
       <c r="G45" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="46" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B46" s="4" t="s">
-        <v>64</v>
+        <v>48</v>
       </c>
       <c r="C46" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D46" s="4"/>
       <c r="E46" s="4">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="F46" s="1"/>
       <c r="G46" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A47" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B47" s="4" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="C47" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D47" s="4"/>
       <c r="E47" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F47" s="1"/>
       <c r="G47" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B48" s="4" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="C48" s="4">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="D48" s="4"/>
       <c r="E48" s="4">
@@ -2476,15 +2580,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A49" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B49" s="4" t="s">
-        <v>68</v>
+        <v>45</v>
       </c>
       <c r="C49" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D49" s="4"/>
       <c r="E49" s="4">
@@ -2495,53 +2599,53 @@
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B50" s="4" t="s">
-        <v>69</v>
+        <v>44</v>
       </c>
       <c r="C50" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D50" s="4"/>
       <c r="E50" s="4">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F50" s="1"/>
       <c r="G50" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="51" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A51" s="4" t="s">
-        <v>67</v>
+        <v>15</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>42</v>
+        <v>72</v>
       </c>
       <c r="C51" s="4">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D51" s="4"/>
       <c r="E51" s="4">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="F51" s="1"/>
       <c r="G51" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="52" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>59</v>
+        <v>71</v>
       </c>
       <c r="C52" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D52" s="4"/>
       <c r="E52" s="4">
@@ -2552,15 +2656,15 @@
         <v>0</v>
       </c>
     </row>
-    <row r="53" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A53" s="4" t="s">
         <v>14</v>
       </c>
       <c r="B53" s="4" t="s">
-        <v>58</v>
+        <v>72</v>
       </c>
       <c r="C53" s="4">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D53" s="4"/>
       <c r="E53" s="4">
@@ -2571,18 +2675,26 @@
         <v>0</v>
       </c>
     </row>
-    <row r="54" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="4"/>
-      <c r="B54" s="4"/>
-      <c r="C54" s="4"/>
+    <row r="54" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A54" s="4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B54" s="4" t="s">
+        <v>80</v>
+      </c>
+      <c r="C54" s="4">
+        <v>3</v>
+      </c>
       <c r="D54" s="4"/>
-      <c r="E54" s="4"/>
+      <c r="E54" s="4">
+        <v>8</v>
+      </c>
       <c r="F54" s="1"/>
       <c r="G54" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="55" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A55" s="4"/>
       <c r="B55" s="4"/>
       <c r="C55" s="4"/>
@@ -2593,7 +2705,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="56" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A56" s="4"/>
       <c r="B56" s="4"/>
       <c r="C56" s="4"/>
@@ -2604,7 +2716,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A57" s="4"/>
       <c r="B57" s="4"/>
       <c r="C57" s="4"/>
@@ -2615,7 +2727,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A58" s="4"/>
       <c r="B58" s="4"/>
       <c r="C58" s="4"/>
@@ -2626,7 +2738,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A59" s="4"/>
       <c r="B59" s="4"/>
       <c r="C59" s="4"/>
@@ -2637,7 +2749,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A60" s="4"/>
       <c r="B60" s="4"/>
       <c r="C60" s="4"/>
@@ -2648,18 +2760,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A61" s="4"/>
       <c r="B61" s="4"/>
       <c r="C61" s="4"/>
       <c r="D61" s="4"/>
       <c r="E61" s="4"/>
-      <c r="F61" s="1"/>
+      <c r="F61" s="4"/>
       <c r="G61" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A62" s="4"/>
       <c r="B62" s="4"/>
       <c r="C62" s="4"/>
@@ -2670,7 +2782,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A63" s="4"/>
       <c r="B63" s="4"/>
       <c r="C63" s="4"/>
@@ -2681,7 +2793,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A64" s="4"/>
       <c r="B64" s="4"/>
       <c r="C64" s="4"/>
@@ -2692,18 +2804,18 @@
         <v>0</v>
       </c>
     </row>
-    <row r="65" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A65" s="4"/>
       <c r="B65" s="4"/>
       <c r="C65" s="4"/>
       <c r="D65" s="4"/>
       <c r="E65" s="4"/>
-      <c r="F65" s="4"/>
+      <c r="F65" s="1"/>
       <c r="G65" s="2" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="66" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A66" s="4"/>
       <c r="B66" s="4"/>
       <c r="C66" s="4"/>
@@ -2714,7 +2826,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="67" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A67" s="4"/>
       <c r="B67" s="4"/>
       <c r="C67" s="4"/>
@@ -2725,66 +2837,14 @@
         <v>0</v>
       </c>
     </row>
-    <row r="68" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A68" s="4"/>
-      <c r="B68" s="4"/>
-      <c r="C68" s="4"/>
-      <c r="D68" s="4"/>
-      <c r="E68" s="4"/>
-      <c r="F68" s="1"/>
-      <c r="G68" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A69" s="4"/>
-      <c r="B69" s="4"/>
-      <c r="C69" s="4"/>
-      <c r="D69" s="4"/>
-      <c r="E69" s="4"/>
-      <c r="F69" s="1"/>
-      <c r="G69" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A70" s="4"/>
-      <c r="B70" s="4"/>
-      <c r="C70" s="4"/>
-      <c r="D70" s="4"/>
-      <c r="E70" s="4"/>
-      <c r="F70" s="1"/>
-      <c r="G70" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" hidden="1" x14ac:dyDescent="0.25">
-      <c r="A71" s="4"/>
-      <c r="B71" s="4"/>
-      <c r="C71" s="4"/>
-      <c r="D71" s="4"/>
-      <c r="E71" s="4"/>
-      <c r="F71" s="1"/>
-      <c r="G71" s="2" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="E75" s="5">
-        <f>SUBTOTAL(9,E9:E19)</f>
-        <v>10</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:G71" xr:uid="{515B20D0-7813-4B7C-85BE-27293B2A524B}">
+  <autoFilter ref="A1:G67" xr:uid="{515B20D0-7813-4B7C-85BE-27293B2A524B}">
     <filterColumn colId="2">
-      <filters>
-        <filter val="0"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="6">
-      <filters>
-        <filter val="FAUX"/>
+      <filters blank="1">
+        <filter val="1"/>
+        <filter val="2"/>
+        <filter val="3"/>
+        <filter val="4"/>
       </filters>
     </filterColumn>
   </autoFilter>
@@ -2796,13 +2856,13 @@
           <x14:formula1>
             <xm:f>dashboard!$B$3:$B$9</xm:f>
           </x14:formula1>
-          <xm:sqref>A2:A7 A52:A53 A43:A50 A9:A40</xm:sqref>
+          <xm:sqref>A2:A7 A9:A37 A41:A54</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E11CFFA5-4840-4999-8AA4-19C490454A05}">
           <x14:formula1>
             <xm:f>dashboard!$B$3:$B$10</xm:f>
           </x14:formula1>
-          <xm:sqref>A8 A51 A41:A42</xm:sqref>
+          <xm:sqref>A8 A38:A40</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>